<commit_message>
Saathi Platform Stabilization v121.0 - Zero-Echo Generation & Raw-Mode Code Drafting
</commit_message>
<xml_diff>
--- a/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
+++ b/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4c0d8e52-4fc1-4552-9d8b-42a2e463d1f7</t>
+          <t>7a1ecdd3-24b7-4a12-9aad-a477268c2131</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello there</t>
+          <t>Hello</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-22T01:19:34.320774+00:00</t>
+          <t>2026-04-22T03:15:31.262087+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22T02:01:04.193197+00:00</t>
+          <t>2026-04-22T03:15:51.263162+00:00</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,12 +679,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bf421e86-c314-4fca-b76d-bc2223d4c55b</t>
+          <t>0ac113fd-76a8-458c-bc26-4be0d2f7399f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4c0d8e52-4fc1-4552-9d8b-42a2e463d1f7</t>
+          <t>7a1ecdd3-24b7-4a12-9aad-a477268c2131</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -699,45 +699,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hello there</t>
+          <t>Hello</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-04-22T02:01:04.193197+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ee0d4fa7-38ea-494b-92d4-8b4e403c2f17</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>4c0d8e52-4fc1-4552-9d8b-42a2e463d1f7</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>sharonmelhi365_gmail_com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saathi hit a routing error: NEURAL CORE INSTABILITY: All providers failed. Last Error: Groq connection failed: Groq 413: {"error":{"message":"Request too large for model `llama-3.1-8b-instant` in organization `org_01kjm3waf2e14tjx5gj0fb33ya` service tier `on_demand` on tokens per minute (TPM): Limit 6000, Requested 8380, please reduce your message size and try again. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"tokens","code":"rate_limit_exceeded"}}
-</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-04-22T02:01:06.308514+00:00</t>
+          <t>2026-04-22T03:15:51.263162+00:00</t>
         </is>
       </c>
     </row>
@@ -810,7 +777,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ya29.a0Aa7MYipveycyPMI6cEyNoASSibDNhCLc3Q-1nmBAzSNzvt7k_ZiWVCoYK_GbaSG_wanzHDN9E9DPyKCoiETKZD63-ikpCkLH2bXhtADlrY1b8HbGvBfo4lB05rY_MUgTmrAEjNpRqNxf4PGmracJkaaHG_SWdY0RA2gbjqFVikn3XMl01t3kxsWHtD88PkoYd3V_KIwaCgYKAcISARUSFQHGX2MiHUvMnKp-_4sLauFh1Vzjlg0206</t>
+          <t>ya29.a0Aa7MYiqwijuV7LUImSets01LEstiW2FVlkOSQ2goIVlp6iibEINMyIZbSuU_EAcvxt3mr5lZQH02WeRNDtkQZEmDnfCYyczdUSKP4oyrMRYTYJKHhVWFABd_NlTfbiGcm03oVmKEmAKTtBeaHcFCI7YNlT4jUwucysYowVlU6iO0EKbn6px3KSSmKd6p7GLxQUykkuMaCgYKAb0SARUSFQHGX2Miouvn6NM3iuFWyLPnQBy8Ow0206</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -820,7 +787,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22T02:19:28.823909+00:00</t>
+          <t>2026-04-22T03:36:21.386275+00:00</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -835,7 +802,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-04-22T02:07:20.162269+00:00</t>
+          <t>2026-04-22T03:20:07.522629+00:00</t>
         </is>
       </c>
     </row>
@@ -901,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1020,6 +987,57 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>2026-04-22T01:27:35.149147+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>45626bb9-cdbe-42ae-bd9a-478399d43311</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOCUMENT SUMMARY [Polyglot: sections_8_11_final.docx]: ஸ்மார்ட் வாட்டர் தரக் கண்காணிப்பு: ஒரு இலக்கிய ஆய்வு
+(பிரிவு 8–11)
+8. ஸ்மார்ட் வாட்டர் கண்காணிப்பின் வழக்கு ஆய்வுகள்
+AI-IoT நீர் கண்காணிப்பின் நடைமுறை ஆதாயங்கள் மற்றும் தொடர்ச்சியான தடைகள் இரண்டையும் நான்கு சூழல்களில் களப் வரிசைப்படுத்தல்கள் விளக்குகின்றன. யாங்சே ஆற்றில், லியு மற்றும் பலர். இரண்டரை ஆண்டுகளில் [CS1] 30 நிமிட இடைவெளியில் கரைந்த ஆக்ஸிஜன், pH, கொந்தளிப்பு, அம்மோனியா-நைட்ரஜன் மற்றும் COD ஆகியவற்றைப் பதிவுசெய்யும் IoT சென்சார்கள் கொண்ட ஒரு தானியங்கி கண்காணிப்பு நிலையம் பொருத்தப்பட்டுள்ளது. இந்த தொடர்ச்சியான ஸ்ட்ரீமில் பயிற்சியளிக்கப்பட்ட LSTM ஆனது ஆறு மாதங்களுக்கு முன்பே 0.043 mg/L RMSE உடன் கரைந்த ஆக்ஸிஜனைக் கணித்துள்ளது, இது வழக்கமான பின்-பரப்பு நெட்வொர்க்குகளை 23% விஞ்சியது - இதன் விளைவாக அவ்வப்போது கிராப் மாதிரி மூலம் அடைய முடியாது. கழிவுநீர் துறையில், சீன WWTP பைலட்டிடம் பயன்படுத்தப்பட்ட தனிமைப்படுத்தப்பட்ட காடு மற்றும் ANN காற்றோட்டக் கட்டுப்படுத்தி ஆற்றல் நுகர்வு 14% குறைக்கப்பட்டது மற்றும் மூன்று நிமிடங்களுக்குள் முரண்பாடான செல்வாக்கு பருப்புகளைக் கண்டறிந்து, [CS3] ச</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-04-22T02:54:01.606028+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3f616a63-2d74-4df0-9813-300e62c86072</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOCUMENT SUMMARY [Polyglot: sections_4_6_final.docx]: ਸਮਾਰਟ ਵਾਟਰ ਕੁਆਲਿਟੀ ਮਾਨੀਟਰਿੰਗ: ਆਈਓਟੀ ਆਰਕੀਟੈਕਚਰ, ਆਰਟੀਫੀਸ਼ੀਅਲ ਇੰਟੈਲੀਜੈਂਸ ਵਿਧੀਆਂ, ਅਤੇ ਏਕੀਕ੍ਰਿਤ AIoT ਪ੍ਰਣਾਲੀਆਂ ਦੀ ਇੱਕ ਸਾਹਿਤ ਸਮੀਖਿਆ
+(ਕੰਪਿਊਟਰ ਸਾਇੰਸ ਕੰਪੋਨੈਂਟ — ਸੈਕਸ਼ਨ 4, 5, ਅਤੇ 6)
+ਕੀਵਰਡਸ: ਚੀਜ਼ਾਂ ਦਾ ਇੰਟਰਨੈਟ, ਪਾਣੀ ਦੀ ਗੁਣਵੱਤਾ ਦੀ ਨਿਗਰਾਨੀ, ਮਸ਼ੀਨ ਸਿਖਲਾਈ, ਡੂੰਘੀ ਸਿਖਲਾਈ, ਐਲਐਸਟੀਐਮ, ਵਿਗਾੜ ਖੋਜ, ਏ.ਆਈ.ਓ.ਟੀ.
+4. ਪਾਣੀ ਦੀ ਗੁਣਵੱਤਾ ਦੀ ਨਿਗਰਾਨੀ ਵਿੱਚ ਚੀਜ਼ਾਂ ਦਾ ਇੰਟਰਨੈਟ (IoT)
+ਪਰੰਪਰਾਗਤ ਪਾਣੀ ਦੀ ਗੁਣਵੱਤਾ ਦੀ ਨਿਗਰਾਨੀ ਪ੍ਰਯੋਗਸ਼ਾਲਾ ਦੇ ਵਿਸ਼ਲੇਸ਼ਣ ਤੋਂ ਬਾਅਦ ਡਿਸਕਰੀਟ ਗ੍ਰੈਬ ਸੈਂਪਲਿੰਗ 'ਤੇ ਨਿਰਭਰ ਕਰਦੀ ਹੈ, ਇੱਕ ਪ੍ਰਕਿਰਿਆ ਜੋ 24 ਤੋਂ 96 ਘੰਟਿਆਂ ਦੀ ਡਾਟਾ ਲੇਟੈਂਸੀ ਨੂੰ ਪੇਸ਼ ਕਰਦੀ ਹੈ ਅਤੇ ਅਸਥਾਈ ਗੰਦਗੀ ਦੀਆਂ ਘਟਨਾਵਾਂ ਦਾ ਪਤਾ ਨਹੀਂ ਲਗਾ ਸਕਦੀ। IoT-ਅਧਾਰਿਤ ਨਿਗਰਾਨੀ ਪੂਰੇ ਪਾਣੀ ਦੇ ਵਾਤਾਵਰਣ ਵਿੱਚ ਆਟੋਨੋਮਸ ਸੈਂਸਿੰਗ ਨੋਡਾਂ ਨੂੰ ਵੰਡ ਕੇ, ਲਗਾਤਾਰ ਮਲਟੀਵੈਰੀਏਟ ਮਾਪ ਅਤੇ ਵਿਸ਼ਲੇਸ਼ਣਾਤਮਕ ਪਲੇਟਫਾਰਮਾਂ ਦੇ ਨੇੜੇ-ਅਸਲ-ਟਾਈਮ ਪ੍ਰਸਾਰਣ ਨੂੰ ਸਮਰੱਥ ਬਣਾ ਕੇ ਇਸ ਅੰਤਰ ਨੂੰ ਹੱਲ ਕਰਦੀ ਹੈ। ਜੱਬਾਰ ਆਦਿ। ਨੇ ਦਿਖਾਇਆ ਕਿ LoRaWAN-ਕਨੈਕਟਡ IoT ਨੋਡ ਸੈਲੂਲਰ ਬੁਨਿਆਦੀ ਢਾਂਚੇ [CS6] ਦੀ ਲਾਗਤ ਦੇ ਇੱਕ ਹਿੱਸੇ 'ਤੇ ਭੂਗੋਲਿਕ ਤੌਰ 'ਤੇ ਫੈਲੀਆਂ ਸਾਈਟਾਂ ਤੋਂ ਭਰੋਸੇਯੋਗ ਟੈਲੀਮੈਟਰੀ ਨੂੰ ਕਾਇਮ ਰੱਖਦੇ ਹਨ, ਜਦਕਿ ਰਹਿਮਾਨੀਅਨ ਐਟ ਅਲ. 87 ਸਮੀਖਿਆ ਕੀਤੇ IoT ਵਾਟਰ ਮਾਨੀਟਰਿੰਗ ਸ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-04-22T03:18:58.490586+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saathi V124.0 - UI/UX Refinement: Polish, Formatting & Pure Chat
</commit_message>
<xml_diff>
--- a/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
+++ b/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7a1ecdd3-24b7-4a12-9aad-a477268c2131</t>
+          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -558,17 +558,98 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello</t>
+          <t>hey</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-22T03:15:31.262087+00:00</t>
+          <t>2026-04-22T04:23:01.997457+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22T03:15:51.263162+00:00</t>
+          <t>2026-04-22T04:57:04.710799+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>d8f152eb-7f36-4c67-973f-b22026c318b5</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>New Thought</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:41:28.365884+00:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:41:28.365884+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3c9e29fa-fa44-4769-812a-5d6ff28c9ab7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>New Thought</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:44:46.575188+00:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:44:46.575188+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bf209789-a072-4a9e-a381-cc0183522724</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>New Thought</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:54:07.215800+00:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:54:07.215800+00:00</t>
         </is>
       </c>
     </row>
@@ -583,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,12 +760,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0ac113fd-76a8-458c-bc26-4be0d2f7399f</t>
+          <t>6f1e4ca6-cf8f-4ef1-a114-826f380bac31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7a1ecdd3-24b7-4a12-9aad-a477268c2131</t>
+          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -699,12 +780,44 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hello</t>
+          <t>hey</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-04-22T03:15:51.263162+00:00</t>
+          <t>2026-04-22T04:57:04.710799+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>f814d7be-f8f6-412d-aa79-4f49060c5c69</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:57:07.890330+00:00</t>
         </is>
       </c>
     </row>
@@ -777,7 +890,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ya29.a0Aa7MYiqwijuV7LUImSets01LEstiW2FVlkOSQ2goIVlp6iibEINMyIZbSuU_EAcvxt3mr5lZQH02WeRNDtkQZEmDnfCYyczdUSKP4oyrMRYTYJKHhVWFABd_NlTfbiGcm03oVmKEmAKTtBeaHcFCI7YNlT4jUwucysYowVlU6iO0EKbn6px3KSSmKd6p7GLxQUykkuMaCgYKAb0SARUSFQHGX2Miouvn6NM3iuFWyLPnQBy8Ow0206</t>
+          <t>ya29.a0Aa7MYip2LjhTQ0BDPmuFajzc2gA2PXtDWpvv4qBeqqbO0mJ2wULjkiKisKgx2pDq29c_ClFJ5RLsQ94JW6TSRRyy5EAf6Ero9NtmJFUSXecHxxO4Czje6xtNxkj5h44BbkznOf2uakE-1M9NzzrXsecfcHnE0Sf6_IkbWK3hS1yGfbR5lVEQstczvuQ6Va_5rX70z8cfaCgYKARgSARUSFQHGX2MiNN3JmyEjMVfffcr6hv4kOw0207</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -787,7 +900,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22T03:36:21.386275+00:00</t>
+          <t>2026-04-22T05:56:53.572456+00:00</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -802,7 +915,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-04-22T03:20:07.522629+00:00</t>
+          <t>2026-04-22T04:57:08.055774+00:00</t>
         </is>
       </c>
     </row>
@@ -868,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1038,6 +1151,102 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>2026-04-22T03:18:58.490586+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>25f14d99-3656-408a-8434-04fa57094a8f</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOCUMENT SUMMARY [Polyglot: causal_clf_blueprint.docx]: ग्राफ-निर्देशित कारण धारणा
+मजबूत दृश्य-मोटर नियंत्रण के लिए
+संपूर्ण शोध खाका, साहित्य समीक्षा और कार्यान्वयन योजना
+लेखक: शेरोन मेलही (सीएस/एआई लीड) |  ख़ुशी (रोबोटिक्स लीड)
+पर्यवेक्षक: के.एस. स्वार्नालाथा
+एमिटी स्कूल ऑफ इंजीनियरिंग एंड टेक्नोलॉजी, एमिटी यूनिवर्सिटी बेंगलुरु
+लक्ष्य स्थान: भारतीय नियंत्रण सम्मेलन (आईसीसी) 2025 | जर्नल एक्सटेंशन: नियंत्रण प्रणाली प्रौद्योगिकी पर आईईईई लेनदेन
+0. सरल व्याख्या (ELI5 - पहले इसे पढ़ें)
+समीकरणों में गोता लगाने से पहले, यहां बताया गया है कि यह पेपर वास्तव में क्या करता है, स्पष्ट रूप से समझाया गया है।
+0.1 हम किस समस्या का समाधान कर रहे हैं?
+कल्पना कीजिए कि आप एक रोबोट (ड्रोन, पहिएदार रोबोट, सर्जिकल आर्म) को कैमरे का उपयोग करके नेविगेट करने का प्रशिक्षण दे रहे हैं। आप इसे एक अनुरूपित वातावरण में प्रशिक्षित करते हैं जो पर्यावरण ए जैसा दिखता है: उज्ज्वल धूप वाला दिन, स्पष्ट बनावट, नीला आकाश। रोबोट पूरी तरह से उड़ना सीखता है। फिर आप पर्यावरण बी पर स्विच करते हैं: बादल छाए हुए, धूमिल, अलग-अलग इलाके की बनावट। रोबोट क्रैश हो गया. क्यों? क्योंकि कैम</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:32:02.470797+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6e1294b8-863c-43d3-8ad6-66b05a4a71d2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOCUMENT SUMMARY [Polyglot: causal_clf_blueprint.docx]: గ్రాఫ్-గైడెడ్ కాజుల్ పర్సెప్షన్
+బలమైన విజువల్-మోటార్ నియంత్రణ కోసం
+పూర్తి రీసెర్చ్ బ్లూప్రింట్, లిటరేచర్ రివ్యూ &amp; ఇంప్లిమెంటేషన్ ప్లాన్
+రచయితలు: షారన్ మెల్హి (CS/AI లీడ్) |  ఖుషీ (రోబోటిక్స్ లీడ్)
+సూపర్‌వైజర్: కె.ఎస్. స్వర్ణలత
+అమిటీ స్కూల్ ఆఫ్ ఇంజనీరింగ్ అండ్ టెక్నాలజీ, అమిటీ యూనివర్సిటీ బెంగళూరు
+లక్ష్య వేదిక: ఇండియన్ కంట్రోల్ కాన్ఫరెన్స్ (ICC) 2025 | జర్నల్ ఎక్స్‌టెన్షన్: కంట్రోల్ సిస్టమ్స్ టెక్నాలజీపై IEEE లావాదేవీలు
+0. సాధారణ వివరణ (ELI5 — దీన్ని ముందుగా చదవండి)
+సమీకరణాలలోకి ప్రవేశించే ముందు, ఈ కాగితం ఏమి చేస్తుందో ఇక్కడ స్పష్టంగా వివరించబడింది.
+0.1 మనం ఏ సమస్యను పరిష్కరిస్తున్నాము?
+మీరు కెమెరాను ఉపయోగించి నావిగేట్ చేయడానికి రోబోట్ (డ్రోన్, వీల్డ్ రోబోట్, సర్జికల్ ఆర్మ్)కి శిక్షణ ఇస్తున్నారని ఊహించుకోండి. మీరు పర్యావరణం A వలె కనిపించే అనుకరణ వాతావరణంలో శిక్షణనిస్తారు: ప్రకాశవంతమైన ఎండ, స్పష్టమైన అల్లికలు, నీలి ఆకాశం. రోబోట్ ఖచ్చితంగా ఎగరడం నేర్చుకుంటుంది. అప్పుడు మీరు పర్యావరణం Bకి మారండి: మేఘావృతమైన, పొగమంచు, విభిన్న భూభాగ అల్లికలు. రోబో క్రాష్ అవుతుంది. ఎందుకు? ఎందుకంటే కెమెరా</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:45:59.682408+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>90ae6192-cee1-4e3f-8650-87ba748f85e1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sharonmelhi365_gmail_com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DOCUMENT SUMMARY [Polyglot: causal_clf_blueprint.docx]: ग्राफ-निर्देशित कारण धारणा
+मजबूत दृश्य-मोटर नियंत्रण के लिए
+संपूर्ण शोध खाका, साहित्य समीक्षा और कार्यान्वयन योजना
+लेखक: शेरोन मेलही (सीएस/एआई लीड) |  ख़ुशी (रोबोटिक्स लीड)
+पर्यवेक्षक: के.एस. स्वार्नालाथा
+एमिटी स्कूल ऑफ इंजीनियरिंग एंड टेक्नोलॉजी, एमिटी यूनिवर्सिटी बेंगलुरु
+लक्ष्य स्थान: भारतीय नियंत्रण सम्मेलन (आईसीसी) 2025 | जर्नल एक्सटेंशन: नियंत्रण प्रणाली प्रौद्योगिकी पर आईईईई लेनदेन
+0. सरल व्याख्या (ELI5 - पहले इसे पढ़ें)
+समीकरणों में गोता लगाने से पहले, यहां बताया गया है कि यह पेपर वास्तव में क्या करता है, स्पष्ट रूप से समझाया गया है।
+0.1 हम किस समस्या का समाधान कर रहे हैं?
+कल्पना कीजिए कि आप एक रोबोट (ड्रोन, पहिएदार रोबोट, सर्जिकल आर्म) को कैमरे का उपयोग करके नेविगेट करने का प्रशिक्षण दे रहे हैं। आप इसे एक अनुरूपित वातावरण में प्रशिक्षित करते हैं जो पर्यावरण ए जैसा दिखता है: उज्ज्वल धूप वाला दिन, स्पष्ट बनावट, नीला आकाश। रोबोट पूरी तरह से उड़ना सीखता है। फिर आप पर्यावरण बी पर स्विच करते हैं: बादल छाए हुए, धूमिल, अलग-अलग इलाके की बनावट। रोबोट क्रैश हो गया. क्यों? क्योंकि कैम</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-04-22T04:46:06.611025+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saathi V125.0 - Outline-First Google Doc Generation (Numbered & Alphabetical)
</commit_message>
<xml_diff>
--- a/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
+++ b/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,7 +575,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>d8f152eb-7f36-4c67-973f-b22026c318b5</t>
+          <t>4efa6df1-732f-425c-bc12-4f262a82f565</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -590,19 +590,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-04-22T04:41:28.365884+00:00</t>
+          <t>2026-04-22T05:03:17.814002+00:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-22T04:41:28.365884+00:00</t>
+          <t>2026-04-22T05:03:17.814002+00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3c9e29fa-fa44-4769-812a-5d6ff28c9ab7</t>
+          <t>619b3573-67fd-41c0-9851-c897370db727</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -617,39 +617,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-04-22T04:44:46.575188+00:00</t>
+          <t>2026-04-22T05:09:21.950177+00:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-04-22T04:44:46.575188+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>bf209789-a072-4a9e-a381-cc0183522724</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>sharonmelhi365_gmail_com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>New Thought</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-04-22T04:54:07.215800+00:00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-04-22T04:54:07.215800+00:00</t>
+          <t>2026-04-22T05:09:21.950177+00:00</t>
         </is>
       </c>
     </row>
@@ -915,7 +888,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-04-22T04:57:08.055774+00:00</t>
+          <t>2026-04-22T05:03:46.991418+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Saathi V126.0 - Absolute Content Purifier (Setext & Greedy Marker Stripping)
</commit_message>
<xml_diff>
--- a/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
+++ b/saathi-api/user_vaults/saathi_storage_sharonmelhi365_gmail_com.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
+          <t>619b3573-67fd-41c0-9851-c897370db727</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -558,24 +558,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hey</t>
+          <t>New Thought</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-22T04:23:01.997457+00:00</t>
+          <t>2026-04-22T05:09:21.950177+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-04-22T04:57:04.710799+00:00</t>
+          <t>2026-04-22T05:09:21.950177+00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4efa6df1-732f-425c-bc12-4f262a82f565</t>
+          <t>8c79b997-ebcf-4119-97f9-0cb3bf938cad</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -590,39 +590,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-04-22T05:03:17.814002+00:00</t>
+          <t>2026-04-22T05:12:03.079614+00:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-22T05:03:17.814002+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>619b3573-67fd-41c0-9851-c897370db727</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>sharonmelhi365_gmail_com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>New Thought</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-04-22T05:09:21.950177+00:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-04-22T05:09:21.950177+00:00</t>
+          <t>2026-04-22T05:12:03.079614+00:00</t>
         </is>
       </c>
     </row>
@@ -637,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,70 +703,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>6f1e4ca6-cf8f-4ef1-a114-826f380bac31</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>sharonmelhi365_gmail_com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>hey</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-04-22T04:57:04.710799+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>f814d7be-f8f6-412d-aa79-4f49060c5c69</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>7e86290a-328b-490d-99f2-98826f638f1b</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>sharonmelhi365_gmail_com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>hello</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-04-22T04:57:07.890330+00:00</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -888,7 +797,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-04-22T05:03:46.991418+00:00</t>
+          <t>2026-04-22T05:12:42.356378+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>